<commit_message>
Laminas regeneradas, informes reconstruidos y baja de laminas_comunales
</commit_message>
<xml_diff>
--- a/output/graficos_nacionales/plot_nacional_d_apoyopot_a_2018.xlsx
+++ b/output/graficos_nacionales/plot_nacional_d_apoyopot_a_2018.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="729">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="732">
   <si>
     <t xml:space="preserve">year</t>
   </si>
@@ -2167,7 +2167,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-07-27 22:02</t>
+    <t xml:space="preserve">2026-09-07 12:42</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -2179,16 +2179,25 @@
     <t xml:space="preserve">Imagen asociada</t>
   </si>
   <si>
-    <t xml:space="preserve"/>
+    <t xml:space="preserve">plot_nacional_d_apoyopot_a_2018.png</t>
   </si>
   <si>
     <t xml:space="preserve">Indicador</t>
   </si>
   <si>
+    <t xml:space="preserve">Otras relaciones demográficas</t>
+  </si>
+  <si>
     <t xml:space="preserve">Unidad territorial</t>
   </si>
   <si>
+    <t xml:space="preserve">Comuna (vista nacional macrozonal)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2018</t>
   </si>
   <si>
     <t xml:space="preserve">variable</t>
@@ -13577,23 +13586,23 @@
         <v>721</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>720</v>
+        <v>726</v>
       </c>
     </row>
   </sheetData>
@@ -13615,21 +13624,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>725</v>
+        <v>728</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>727</v>
+        <v>730</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>15</v>
@@ -13638,7 +13647,7 @@
         <v>2018</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
     </row>
   </sheetData>

</xml_diff>